<commit_message>
fix(catalog): isolate supplier update test with tempfile so production catalogo_actualizado.xlsx is never truncated
</commit_message>
<xml_diff>
--- a/assets/catalogo_actualizado.xlsx
+++ b/assets/catalogo_actualizado.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -497,7 +497,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ART01</t>
+          <t>ART001</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -507,11 +507,11 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Caja x 6</t>
+          <t>Caja x 6 u.</t>
         </is>
       </c>
       <c r="D2" s="4" t="n">
-        <v>16200</v>
+        <v>14400</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
@@ -527,7 +527,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>ART02</t>
+          <t>ART002</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -537,11 +537,11 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Fardo x 10</t>
+          <t>Fardo x 10 u.</t>
         </is>
       </c>
       <c r="D3" s="4" t="n">
-        <v>13900</v>
+        <v>12500</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
@@ -557,21 +557,21 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>ART03</t>
+          <t>ART003</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Coca Cola 2.25L</t>
+          <t>Arroz Lucchetti Largo Fino 1kg</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Pack x 6</t>
+          <t>Fardo x 10 u.</t>
         </is>
       </c>
       <c r="D4" s="4" t="n">
-        <v>21500</v>
+        <v>16000</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
@@ -580,7 +580,367 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
+          <t>Almacén</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>ART004</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Fideos Matarazzo Guiseros 500g</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Caja x 15 u.</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>18000</v>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Almacén</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>ART005</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Azúcar Ledesma Clásica 1kg</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Fardo x 10 u.</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>11000</v>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Almacén</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>ART006</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Puré de Tomate De Cecco 520g</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Caja x 12 u.</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>9800</v>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Almacén</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>ART007</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Queso Cremoso La Paulina</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Horma x 4kg</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>28000</v>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Lácteos y Fríos</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>ART008</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Leche Entera La Serenísima 1L</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Caja x 12 u.</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>15600</v>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Lácteos y Fríos</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>ART009</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Yogur Firme Ilolay 120g</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Pack x 8 u.</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>6400</v>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Lácteos y Fríos</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>ART010</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Gaseosa Coca Cola 2.25L</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Pack x 6 u.</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>19200</v>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
           <t>Bebidas</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>ART011</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Cerveza Quilmes Clásica 1L</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Cajón x 12 u.</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>24000</v>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Bebidas</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>ART012</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Agua Mineral Villavicencio 2L</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Pack x 6 u.</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>8400</v>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Bebidas</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>ART013</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Yerba Playadito 1kg</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Fardo x 10 u.</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>38000</v>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Almacén</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>ART014</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Galletitas Oreo 118g</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Caja x 24 u.</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>26400</v>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Golosinas</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>ART015</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Mayonesa Hellmanns Doypack 475g</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Caja x 12 u.</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>17500</v>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Almacén</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: auto-export Excel file on preset rubro switch so physical file is always ready for live client demos
</commit_message>
<xml_diff>
--- a/assets/catalogo_actualizado.xlsx
+++ b/assets/catalogo_actualizado.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -497,21 +497,21 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ART001</t>
+          <t>ART-001</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Aceite Cañuelas 1.5L</t>
+          <t>Tornillos autoperforantes 1 pulgada</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Caja x 6 u.</t>
+          <t>Caja x 1000</t>
         </is>
       </c>
       <c r="D2" s="4" t="n">
-        <v>14400</v>
+        <v>8500</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
@@ -520,28 +520,28 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Almacén</t>
+          <t>Tornillería</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>ART002</t>
+          <t>ART-002</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Harina Pureza 000 1kg</t>
+          <t>Tornillos tirafondo 1/4 x 2</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Fardo x 10 u.</t>
+          <t>Caja x 100</t>
         </is>
       </c>
       <c r="D3" s="4" t="n">
-        <v>12500</v>
+        <v>7200</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
@@ -550,28 +550,28 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Almacén</t>
+          <t>Tornillería</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>ART003</t>
+          <t>ART-003</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Arroz Lucchetti Largo Fino 1kg</t>
+          <t>Tarugos con tope N°8</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Fardo x 10 u.</t>
+          <t>Bolsa x 100</t>
         </is>
       </c>
       <c r="D4" s="4" t="n">
-        <v>16000</v>
+        <v>3200</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
@@ -580,28 +580,28 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Almacén</t>
+          <t>Fijación</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>ART004</t>
+          <t>ART-004</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Fideos Matarazzo Guiseros 500g</t>
+          <t>Disco de corte amoladora 115mm x 1mm</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Caja x 15 u.</t>
+          <t>Unidad</t>
         </is>
       </c>
       <c r="D5" s="4" t="n">
-        <v>18000</v>
+        <v>1400</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
@@ -610,28 +610,28 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Almacén</t>
+          <t>Abrasivos</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>ART005</t>
+          <t>ART-005</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Azúcar Ledesma Clásica 1kg</t>
+          <t>Disco de desbaste metal 115mm</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Fardo x 10 u.</t>
+          <t>Unidad</t>
         </is>
       </c>
       <c r="D6" s="4" t="n">
-        <v>11000</v>
+        <v>2800</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
@@ -640,28 +640,28 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Almacén</t>
+          <t>Abrasivos</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>ART006</t>
+          <t>ART-006</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Puré de Tomate De Cecco 520g</t>
+          <t>Disco diamantado continuo 115mm</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Caja x 12 u.</t>
+          <t>Unidad</t>
         </is>
       </c>
       <c r="D7" s="4" t="n">
-        <v>9800</v>
+        <v>6500</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
@@ -670,28 +670,28 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Almacén</t>
+          <t>Abrasivos</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>ART007</t>
+          <t>ART-007</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Queso Cremoso La Paulina</t>
+          <t>Amoladora angular 115mm 850W</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Horma x 4kg</t>
+          <t>Unidad</t>
         </is>
       </c>
       <c r="D8" s="4" t="n">
-        <v>28000</v>
+        <v>68000</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
@@ -700,28 +700,28 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Lácteos y Fríos</t>
+          <t>Herramientas Eléctricas</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>ART008</t>
+          <t>ART-008</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Leche Entera La Serenísima 1L</t>
+          <t>Taladro percutor 13mm 650W</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Caja x 12 u.</t>
+          <t>Unidad</t>
         </is>
       </c>
       <c r="D9" s="4" t="n">
-        <v>15600</v>
+        <v>74000</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
@@ -730,28 +730,28 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Lácteos y Fríos</t>
+          <t>Herramientas Eléctricas</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>ART009</t>
+          <t>ART-009</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Yogur Firme Ilolay 120g</t>
+          <t>Destornillador Phillips 6x100mm</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Pack x 8 u.</t>
+          <t>Unidad</t>
         </is>
       </c>
       <c r="D10" s="4" t="n">
-        <v>6400</v>
+        <v>4800</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
@@ -760,28 +760,28 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Lácteos y Fríos</t>
+          <t>Herramientas Manuales</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>ART010</t>
+          <t>ART-010</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Gaseosa Coca Cola 2.25L</t>
+          <t>Destornillador Plano 6x100mm</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Pack x 6 u.</t>
+          <t>Unidad</t>
         </is>
       </c>
       <c r="D11" s="4" t="n">
-        <v>19200</v>
+        <v>4500</v>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
@@ -790,28 +790,28 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Bebidas</t>
+          <t>Herramientas Manuales</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>ART011</t>
+          <t>ART-011</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Cerveza Quilmes Clásica 1L</t>
+          <t>Juego de destornilladores x 6 piezas</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Cajón x 12 u.</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="D12" s="4" t="n">
-        <v>24000</v>
+        <v>18500</v>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
@@ -820,28 +820,28 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Bebidas</t>
+          <t>Herramientas Manuales</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>ART012</t>
+          <t>ART-012</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Agua Mineral Villavicencio 2L</t>
+          <t>Martillo galponero mango fibra 500g</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Pack x 6 u.</t>
+          <t>Unidad</t>
         </is>
       </c>
       <c r="D13" s="4" t="n">
-        <v>8400</v>
+        <v>14500</v>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
@@ -850,28 +850,28 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Bebidas</t>
+          <t>Herramientas Manuales</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>ART013</t>
+          <t>ART-013</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Yerba Playadito 1kg</t>
+          <t>Pinza universal 8 pulgadas aislada</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Fardo x 10 u.</t>
+          <t>Unidad</t>
         </is>
       </c>
       <c r="D14" s="4" t="n">
-        <v>38000</v>
+        <v>12500</v>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
@@ -880,58 +880,58 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Almacén</t>
+          <t>Herramientas Manuales</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>ART014</t>
+          <t>ART-014</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Galletitas Oreo 118g</t>
+          <t>Alicate corte diagonal 6 pulgadas</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Caja x 24 u.</t>
+          <t>Unidad</t>
         </is>
       </c>
       <c r="D15" s="4" t="n">
-        <v>26400</v>
+        <v>11000</v>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Golosinas</t>
+          <t>Herramientas Manuales</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>ART015</t>
+          <t>ART-015</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Mayonesa Hellmanns Doypack 475g</t>
+          <t>Llave francesa ajustable 10 pulgadas</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Caja x 12 u.</t>
+          <t>Unidad</t>
         </is>
       </c>
       <c r="D16" s="4" t="n">
-        <v>17500</v>
+        <v>16500</v>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
@@ -940,7 +940,277 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Almacén</t>
+          <t>Herramientas Manuales</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>ART-016</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Cinta aisladora negra 20 metros</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Rollo</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Electricidad</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>ART-017</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Cinta de teflón 3/4 x 20m</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Rollo</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>950</v>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Plomería</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>ART-018</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Thinner estándar 1 litro</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Botella</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>4200</v>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Pinturas &amp; Química</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>ART-019</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Aguarrás mineral 1 litro</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Botella</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>3800</v>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Pinturas &amp; Química</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>ART-020</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Sellador de silicona neutra transparente 280ml</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Tubo</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>6800</v>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Adhesivos &amp; Selladores</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>ART-021</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Pegamento de contacto Poxiran 250cc</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Lata</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="n">
+        <v>5400</v>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Adhesivos &amp; Selladores</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>ART-022</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Candado de bronce 40mm con 3 llaves</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="n">
+        <v>8900</v>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Cerrajería</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>ART-023</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Pintura látex interior blanco 4L</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Balde</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="n">
+        <v>22000</v>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Pinturas &amp; Química</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>ART-024</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Lija al agua grano 180</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Pliego</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="n">
+        <v>650</v>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Abrasivos</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: multi-supplier centralization, autonomous excel parser with Gemini fallback, and supplier replenishment baskets
</commit_message>
<xml_diff>
--- a/assets/catalogo_actualizado.xlsx
+++ b/assets/catalogo_actualizado.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -460,6 +460,7 @@
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -493,6 +494,11 @@
           <t>Categoría</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Proveedor</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -523,6 +529,11 @@
           <t>Tornillería</t>
         </is>
       </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Bulonera del Litoral</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -553,6 +564,11 @@
           <t>Tornillería</t>
         </is>
       </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -583,6 +599,11 @@
           <t>Fijación</t>
         </is>
       </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -613,6 +634,11 @@
           <t>Abrasivos</t>
         </is>
       </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -643,6 +669,11 @@
           <t>Abrasivos</t>
         </is>
       </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -673,6 +704,11 @@
           <t>Abrasivos</t>
         </is>
       </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -703,6 +739,11 @@
           <t>Herramientas Eléctricas</t>
         </is>
       </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -733,6 +774,11 @@
           <t>Herramientas Eléctricas</t>
         </is>
       </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -763,6 +809,11 @@
           <t>Herramientas Manuales</t>
         </is>
       </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -793,6 +844,11 @@
           <t>Herramientas Manuales</t>
         </is>
       </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -823,6 +879,11 @@
           <t>Herramientas Manuales</t>
         </is>
       </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -853,6 +914,11 @@
           <t>Herramientas Manuales</t>
         </is>
       </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -883,6 +949,11 @@
           <t>Herramientas Manuales</t>
         </is>
       </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -913,6 +984,11 @@
           <t>Herramientas Manuales</t>
         </is>
       </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -943,6 +1019,11 @@
           <t>Herramientas Manuales</t>
         </is>
       </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -973,6 +1054,11 @@
           <t>Electricidad</t>
         </is>
       </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1003,6 +1089,11 @@
           <t>Plomería</t>
         </is>
       </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1033,6 +1124,11 @@
           <t>Pinturas &amp; Química</t>
         </is>
       </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1063,6 +1159,11 @@
           <t>Pinturas &amp; Química</t>
         </is>
       </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1093,6 +1194,11 @@
           <t>Adhesivos &amp; Selladores</t>
         </is>
       </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1123,6 +1229,11 @@
           <t>Adhesivos &amp; Selladores</t>
         </is>
       </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1153,6 +1264,11 @@
           <t>Cerrajería</t>
         </is>
       </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1183,6 +1299,11 @@
           <t>Pinturas &amp; Química</t>
         </is>
       </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1211,6 +1332,46 @@
       <c r="F25" s="3" t="inlineStr">
         <is>
           <t>Abrasivos</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>FER-001</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Martillo Galponero 20mm</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="n">
+        <v>19500</v>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Bulonera del Litoral</t>
         </is>
       </c>
     </row>

</xml_diff>